<commit_message>
SSA and Smart Switch references replaced with Ampra (SON codes preserved)
</commit_message>
<xml_diff>
--- a/Ampra_Commission_Tracker.xlsx
+++ b/Ampra_Commission_Tracker.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="440">
   <si>
-    <t xml:space="preserve">SSA Commission Tracker — Team Position</t>
+    <t xml:space="preserve">Ampra Commission Tracker — Team Position</t>
   </si>
   <si>
     <t xml:space="preserve">Positions from 20/07/26 onward · HubSpot pull 25/08/26 · ad spend to 20/08/26 · All pending deals are based on cash amounts and may change with finance and ACP charges.</t>
@@ -1277,7 +1277,7 @@
     <t xml:space="preserve">READ ME</t>
   </si>
   <si>
-    <t xml:space="preserve">SSA Commission Tracker · pull 25/08/26</t>
+    <t xml:space="preserve">Ampra Commission Tracker · pull 25/08/26</t>
   </si>
   <si>
     <t xml:space="preserve">Who is tracked</t>
@@ -2013,7 +2013,7 @@
         <v>-6370.33</v>
       </c>
       <c r="G5" s="4" t="str">
-        <f aca="false">IF(F5&gt;=0,"SSA OWES","TO EARN BACK")</f>
+        <f aca="false">IF(F5&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
         <v>TO EARN BACK</v>
       </c>
       <c r="H5" s="5" t="n">
@@ -2024,8 +2024,8 @@
         <v>2293.97</v>
       </c>
       <c r="J5" s="4" t="str">
-        <f aca="false">IF(I5&gt;=0,"SSA OWES","TO EARN BACK")</f>
-        <v>SSA OWES</v>
+        <f aca="false">IF(I5&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
+        <v>AMPRA OWES</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2049,7 +2049,7 @@
         <v>-4095.82</v>
       </c>
       <c r="G6" s="4" t="str">
-        <f aca="false">IF(F6&gt;=0,"SSA OWES","TO EARN BACK")</f>
+        <f aca="false">IF(F6&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
         <v>TO EARN BACK</v>
       </c>
       <c r="H6" s="5" t="n">
@@ -2060,7 +2060,7 @@
         <v>-824.3</v>
       </c>
       <c r="J6" s="4" t="str">
-        <f aca="false">IF(I6&gt;=0,"SSA OWES","TO EARN BACK")</f>
+        <f aca="false">IF(I6&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
         <v>TO EARN BACK</v>
       </c>
     </row>
@@ -2085,8 +2085,8 @@
         <v>686.13</v>
       </c>
       <c r="G7" s="4" t="str">
-        <f aca="false">IF(F7&gt;=0,"SSA OWES","TO EARN BACK")</f>
-        <v>SSA OWES</v>
+        <f aca="false">IF(F7&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
+        <v>AMPRA OWES</v>
       </c>
       <c r="H7" s="5" t="n">
         <v>11804.4</v>
@@ -2096,8 +2096,8 @@
         <v>12490.53</v>
       </c>
       <c r="J7" s="4" t="str">
-        <f aca="false">IF(I7&gt;=0,"SSA OWES","TO EARN BACK")</f>
-        <v>SSA OWES</v>
+        <f aca="false">IF(I7&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
+        <v>AMPRA OWES</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2121,7 +2121,7 @@
         <v>-3300.01</v>
       </c>
       <c r="G8" s="4" t="str">
-        <f aca="false">IF(F8&gt;=0,"SSA OWES","TO EARN BACK")</f>
+        <f aca="false">IF(F8&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
         <v>TO EARN BACK</v>
       </c>
       <c r="H8" s="5" t="n">
@@ -2132,7 +2132,7 @@
         <v>-960.37</v>
       </c>
       <c r="J8" s="4" t="str">
-        <f aca="false">IF(I8&gt;=0,"SSA OWES","TO EARN BACK")</f>
+        <f aca="false">IF(I8&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
         <v>TO EARN BACK</v>
       </c>
     </row>
@@ -2157,8 +2157,8 @@
         <v>0</v>
       </c>
       <c r="G9" s="4" t="str">
-        <f aca="false">IF(F9&gt;=0,"SSA OWES","TO EARN BACK")</f>
-        <v>SSA OWES</v>
+        <f aca="false">IF(F9&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
+        <v>AMPRA OWES</v>
       </c>
       <c r="H9" s="5" t="n">
         <v>615.7</v>
@@ -2168,8 +2168,8 @@
         <v>615.7</v>
       </c>
       <c r="J9" s="4" t="str">
-        <f aca="false">IF(I9&gt;=0,"SSA OWES","TO EARN BACK")</f>
-        <v>SSA OWES</v>
+        <f aca="false">IF(I9&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
+        <v>AMPRA OWES</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2196,7 +2196,7 @@
         <v>-13080.03</v>
       </c>
       <c r="G10" s="7" t="str">
-        <f aca="false">IF(F10&gt;=0,"SSA OWES","TO EARN BACK")</f>
+        <f aca="false">IF(F10&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
         <v>TO EARN BACK</v>
       </c>
       <c r="H10" s="8" t="n">
@@ -2208,8 +2208,8 @@
         <v>13615.53</v>
       </c>
       <c r="J10" s="7" t="str">
-        <f aca="false">IF(I10&gt;=0,"SSA OWES","TO EARN BACK")</f>
-        <v>SSA OWES</v>
+        <f aca="false">IF(I10&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
+        <v>AMPRA OWES</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Joe set to FTE (Salaried) per the people table; Holly confirmed Contractor
</commit_message>
<xml_diff>
--- a/Ampra_Commission_Tracker.xlsx
+++ b/Ampra_Commission_Tracker.xlsx
@@ -74,10 +74,10 @@
     <t xml:space="preserve">Joe</t>
   </si>
   <si>
+    <t xml:space="preserve">Holly</t>
+  </si>
+  <si>
     <t xml:space="preserve">Contractor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holly</t>
   </si>
   <si>
     <t xml:space="preserve">Ollie</t>
@@ -2069,7 +2069,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>0</v>
@@ -2102,10 +2102,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>16</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>0</v>
@@ -2557,7 +2557,7 @@
         <v>35</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>15</v>
@@ -3240,7 +3240,7 @@
         <v>139</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>140</v>
@@ -3260,7 +3260,7 @@
         <v>142</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>140</v>
@@ -3280,7 +3280,7 @@
         <v>143</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>140</v>
@@ -3320,7 +3320,7 @@
         <v>144</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>145</v>
@@ -3340,7 +3340,7 @@
         <v>147</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>140</v>
@@ -3360,7 +3360,7 @@
         <v>147</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>140</v>
@@ -3380,7 +3380,7 @@
         <v>150</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>140</v>
@@ -3400,7 +3400,7 @@
         <v>151</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>140</v>
@@ -3420,7 +3420,7 @@
         <v>152</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>140</v>
@@ -3440,7 +3440,7 @@
         <v>153</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>140</v>
@@ -3460,7 +3460,7 @@
         <v>154</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>140</v>
@@ -3480,7 +3480,7 @@
         <v>155</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>140</v>
@@ -3520,7 +3520,7 @@
         <v>156</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>145</v>
@@ -3540,7 +3540,7 @@
         <v>156</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>140</v>
@@ -3560,7 +3560,7 @@
         <v>157</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>140</v>
@@ -3580,7 +3580,7 @@
         <v>158</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>140</v>
@@ -3600,7 +3600,7 @@
         <v>159</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>140</v>
@@ -3620,7 +3620,7 @@
         <v>160</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>140</v>
@@ -3640,7 +3640,7 @@
         <v>161</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>140</v>
@@ -3660,7 +3660,7 @@
         <v>162</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>140</v>
@@ -3680,7 +3680,7 @@
         <v>163</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>140</v>
@@ -3928,7 +3928,7 @@
         <v>183</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>14</v>
@@ -4090,7 +4090,7 @@
         <v>208</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>15</v>
@@ -4117,7 +4117,7 @@
         <v>211</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>212</v>
@@ -5311,7 +5311,7 @@
         <v>352</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E60" s="4" t="s">
         <v>15</v>
@@ -6012,7 +6012,7 @@
     </row>
     <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B11" s="27" t="s">
         <v>427</v>

</xml_diff>

<commit_message>
Retainers replaced with Scott reconciled Retainer log: Denzel 7500, Hugo 3250
</commit_message>
<xml_diff>
--- a/Ampra_Commission_Tracker.xlsx
+++ b/Ampra_Commission_Tracker.xlsx
@@ -2159,14 +2159,14 @@
         <v>-4789.06</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>5000</v>
+        <v>7500</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>3719.47</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">C5+E5-D5</f>
-        <v>-6069.59</v>
+        <v>-8569.59</v>
       </c>
       <c r="G5" s="4" t="str">
         <f aca="false">IF(F5&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="I5" s="6" t="n">
         <f aca="false">C5+E5+H5-D5</f>
-        <v>14510.46</v>
+        <v>12010.46</v>
       </c>
       <c r="J5" s="4" t="str">
         <f aca="false">IF(I5&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
@@ -2195,14 +2195,14 @@
         <v>-7730.41</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>0</v>
+        <v>3250</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>3715.38</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">C6+E6-D6</f>
-        <v>-4015.03</v>
+        <v>-7265.03</v>
       </c>
       <c r="G6" s="4" t="str">
         <f aca="false">IF(F6&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="I6" s="6" t="n">
         <f aca="false">C6+E6+H6-D6</f>
-        <v>8591.84</v>
+        <v>5341.84</v>
       </c>
       <c r="J6" s="4" t="str">
         <f aca="false">IF(I6&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="D10" s="8" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>9706.25</v>
+        <v>15456.25</v>
       </c>
       <c r="E10" s="8" t="n">
         <f aca="false">SUM(E5:E9)</f>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="F10" s="8" t="n">
         <f aca="false">C10+E10-D10</f>
-        <v>-13193.98</v>
+        <v>-18943.98</v>
       </c>
       <c r="G10" s="7" t="str">
         <f aca="false">IF(F10&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="I10" s="8" t="n">
         <f aca="false">C10+E10+H10-D10</f>
-        <v>39406.01</v>
+        <v>33656.01</v>
       </c>
       <c r="J10" s="7" t="str">
         <f aca="false">IF(I10&gt;=0,"AMPRA OWES","TO EARN BACK")</f>

</xml_diff>

<commit_message>
Ad spend: sales campaigns only - Ampra Job recruitment excluded
</commit_message>
<xml_diff>
--- a/Ampra_Commission_Tracker.xlsx
+++ b/Ampra_Commission_Tracker.xlsx
@@ -2267,14 +2267,14 @@
         <v>0</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>4706.25</v>
+        <v>4659.64</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>903.78</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">C8+E8-D8</f>
-        <v>-3802.47</v>
+        <v>-3755.86</v>
       </c>
       <c r="G8" s="4" t="str">
         <f aca="false">IF(F8&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="I8" s="6" t="n">
         <f aca="false">C8+E8+H8-D8</f>
-        <v>-1259.02</v>
+        <v>-1212.41</v>
       </c>
       <c r="J8" s="4" t="str">
         <f aca="false">IF(I8&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
@@ -2341,7 +2341,7 @@
       </c>
       <c r="D10" s="8" t="n">
         <f aca="false">SUM(D5:D9)</f>
-        <v>15456.25</v>
+        <v>15409.64</v>
       </c>
       <c r="E10" s="8" t="n">
         <f aca="false">SUM(E5:E9)</f>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="F10" s="8" t="n">
         <f aca="false">C10+E10-D10</f>
-        <v>-18943.98</v>
+        <v>-18897.37</v>
       </c>
       <c r="G10" s="7" t="str">
         <f aca="false">IF(F10&gt;=0,"AMPRA OWES","TO EARN BACK")</f>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="I10" s="8" t="n">
         <f aca="false">C10+E10+H10-D10</f>
-        <v>33656.01</v>
+        <v>33702.62</v>
       </c>
       <c r="J10" s="7" t="str">
         <f aca="false">IF(I10&gt;=0,"AMPRA OWES","TO EARN BACK")</f>

</xml_diff>

<commit_message>
Pricing-error adjustments: deduct from the named person after the split, not off the pot
</commit_message>
<xml_diff>
--- a/Ampra_Commission_Tracker.xlsx
+++ b/Ampra_Commission_Tracker.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1256" uniqueCount="476">
   <si>
     <t xml:space="preserve">Ampra Commission Tracker — Team Position</t>
   </si>
@@ -1239,7 +1239,7 @@
     <t xml:space="preserve">75 deals · reference only, not counted in current positions · pull 28/08/26</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimate up to 20/07/26. Figures before that date are reconstructed from HubSpot and contain known inconsistencies — 0 rows flagged below have no install date, no deal value, or no attribution recorded. Commission shown is earned/owed on install, not cash paid. Treat these totals as an estimate for cross-referencing, not a settled ledger.</t>
+    <t xml:space="preserve">Estimate up to 20/07/26. Figures before that date are reconstructed from HubSpot and contain known inconsistencies — 1 rows flagged below have no install date, no deal value, or no attribution recorded. Commission shown is earned/owed on install, not cash paid. Treat these totals as an estimate for cross-referencing, not a settled ledger.</t>
   </si>
   <si>
     <t xml:space="preserve">Formbay +/-</t>
@@ -1324,6 +1324,9 @@
   </si>
   <si>
     <t xml:space="preserve">Fran</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pricing error - $2,500.00 deducted from Denzel</t>
   </si>
   <si>
     <t xml:space="preserve">Beau Jolly</t>
@@ -1665,7 +1668,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1787,6 +1790,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6581,10 +6592,10 @@
         <v>240.29</v>
       </c>
       <c r="J75" s="27" t="n">
-        <v>120.14</v>
+        <v>-1129.86</v>
       </c>
       <c r="K75" s="27" t="n">
-        <v>120.14</v>
+        <v>-1129.86</v>
       </c>
       <c r="L75" s="27" t="n">
         <v>0</v>
@@ -6847,11 +6858,11 @@
       </c>
       <c r="J82" s="8" t="n">
         <f aca="false">SUM(J7:J81)</f>
-        <v>91820.52</v>
+        <v>90570.52</v>
       </c>
       <c r="K82" s="8" t="n">
         <f aca="false">SUM(K7:K81)</f>
-        <v>91820.52</v>
+        <v>90570.52</v>
       </c>
       <c r="L82" s="8" t="n">
         <f aca="false">SUM(L7:L81)</f>
@@ -7825,49 +7836,51 @@
       <c r="O21" s="4"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="11" t="s">
         <v>370</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="12" t="s">
         <v>371</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="12" t="s">
         <v>369</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="12" t="s">
         <v>432</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="G22" s="6" t="n">
+      <c r="G22" s="31" t="n">
         <v>29377</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H22" s="31" t="n">
         <v>27402.91</v>
       </c>
-      <c r="I22" s="6" t="n">
+      <c r="I22" s="31" t="n">
         <v>696.54</v>
       </c>
-      <c r="J22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="6" t="n">
+      <c r="J22" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="31" t="n">
         <v>240.29</v>
       </c>
-      <c r="L22" s="6" t="n">
+      <c r="L22" s="31" t="n">
         <v>-2430.35</v>
       </c>
-      <c r="M22" s="6" t="n">
+      <c r="M22" s="31" t="n">
         <v>240.28</v>
       </c>
-      <c r="N22" s="30" t="s">
+      <c r="N22" s="32" t="s">
         <v>424</v>
       </c>
-      <c r="O22" s="4"/>
+      <c r="O22" s="12" t="s">
+        <v>433</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
@@ -8150,10 +8163,10 @@
         <v>348</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>42</v>
@@ -8285,7 +8298,7 @@
         <v>339</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>15</v>
@@ -8330,7 +8343,7 @@
         <v>336</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>15</v>
@@ -8378,7 +8391,7 @@
         <v>417</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>48</v>
@@ -8420,7 +8433,7 @@
         <v>330</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>417</v>
@@ -8465,10 +8478,10 @@
         <v>330</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>48</v>
@@ -8513,7 +8526,7 @@
         <v>417</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>48</v>
@@ -8555,7 +8568,7 @@
         <v>322</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>417</v>
@@ -8648,7 +8661,7 @@
         <v>417</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>48</v>
@@ -8735,10 +8748,10 @@
         <v>309</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>48</v>
@@ -8780,7 +8793,7 @@
         <v>309</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>15</v>
@@ -8915,10 +8928,10 @@
         <v>301</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>48</v>
@@ -8960,10 +8973,10 @@
         <v>301</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>48</v>
@@ -9005,10 +9018,10 @@
         <v>296</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>48</v>
@@ -9050,10 +9063,10 @@
         <v>296</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>48</v>
@@ -9095,10 +9108,10 @@
         <v>291</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>48</v>
@@ -9140,10 +9153,10 @@
         <v>291</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F51" s="4" t="s">
         <v>48</v>
@@ -9230,10 +9243,10 @@
         <v>285</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>48</v>
@@ -9275,10 +9288,10 @@
         <v>280</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>48</v>
@@ -9320,10 +9333,10 @@
         <v>280</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F55" s="4" t="s">
         <v>48</v>
@@ -9365,10 +9378,10 @@
         <v>275</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F56" s="4" t="s">
         <v>48</v>
@@ -9455,7 +9468,7 @@
         <v>272</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E58" s="4" t="s">
         <v>20</v>
@@ -9500,10 +9513,10 @@
         <v>269</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F59" s="4" t="s">
         <v>42</v>
@@ -9680,10 +9693,10 @@
         <v>257</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F63" s="4" t="s">
         <v>48</v>
@@ -9725,7 +9738,7 @@
         <v>254</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E64" s="4" t="s">
         <v>15</v>
@@ -9770,7 +9783,7 @@
         <v>251</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E65" s="4" t="s">
         <v>15</v>
@@ -9860,7 +9873,7 @@
         <v>245</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E67" s="4" t="s">
         <v>15</v>
@@ -9950,10 +9963,10 @@
         <v>239</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F69" s="4" t="s">
         <v>48</v>
@@ -10085,10 +10098,10 @@
         <v>231</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F72" s="4" t="s">
         <v>48</v>
@@ -10175,7 +10188,7 @@
         <v>226</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E74" s="4" t="s">
         <v>15</v>
@@ -10518,7 +10531,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="20" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -10552,134 +10565,134 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="31" t="s">
-        <v>453</v>
-      </c>
-      <c r="B4" s="32" t="s">
+      <c r="A4" s="33" t="s">
         <v>454</v>
       </c>
+      <c r="B4" s="34" t="s">
+        <v>455</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
-        <v>455</v>
-      </c>
-      <c r="B5" s="32" t="s">
+      <c r="A5" s="33" t="s">
         <v>456</v>
       </c>
+      <c r="B5" s="34" t="s">
+        <v>457</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
-        <v>457</v>
-      </c>
-      <c r="B6" s="32" t="s">
+      <c r="A6" s="33" t="s">
+        <v>458</v>
+      </c>
+      <c r="B6" s="34" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="32" t="s">
-        <v>458</v>
+      <c r="B7" s="34" t="s">
+        <v>459</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="32" t="s">
-        <v>459</v>
+      <c r="B8" s="34" t="s">
+        <v>460</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="32" t="s">
-        <v>460</v>
+      <c r="B9" s="34" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="32" t="s">
-        <v>461</v>
+      <c r="B10" s="34" t="s">
+        <v>462</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="32" t="s">
-        <v>462</v>
+      <c r="B11" s="34" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="31" t="s">
-        <v>463</v>
-      </c>
-      <c r="B12" s="32" t="s">
+      <c r="A12" s="33" t="s">
         <v>464</v>
       </c>
+      <c r="B12" s="34" t="s">
+        <v>465</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
-        <v>465</v>
-      </c>
-      <c r="B13" s="32" t="s">
+      <c r="A13" s="33" t="s">
         <v>466</v>
       </c>
+      <c r="B13" s="34" t="s">
+        <v>467</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
-        <v>467</v>
-      </c>
-      <c r="B14" s="32" t="s">
+      <c r="A14" s="33" t="s">
+        <v>468</v>
+      </c>
+      <c r="B14" s="34" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
-        <v>468</v>
-      </c>
-      <c r="B15" s="32" t="s">
+      <c r="A15" s="33" t="s">
         <v>469</v>
       </c>
+      <c r="B15" s="34" t="s">
+        <v>470</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>470</v>
-      </c>
-      <c r="B16" s="32" t="s">
+      <c r="A16" s="33" t="s">
         <v>471</v>
       </c>
+      <c r="B16" s="34" t="s">
+        <v>472</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
-        <v>472</v>
-      </c>
-      <c r="B17" s="32" t="s">
+      <c r="A17" s="33" t="s">
         <v>473</v>
       </c>
+      <c r="B17" s="34" t="s">
+        <v>474</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="B18" s="32" t="s">
-        <v>474</v>
+      <c r="B18" s="34" t="s">
+        <v>475</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ad spend: recover two unledgered Meta receipts (21/08, 23/08)
A full Gmail sweep with in:anywhere found two AU receipts no previous run had
seen: 21/08 ($149.00 gross, $127.94 chargeable) and 23/08 ($149.00 gross,
$116.59 chargeable), each less its Ampra Job recruitment line. They fill the
ledger's unexplained 20/08 -> 25/08 cadence gap.

Not a dedupe difference: this sweep finds 43 messages / 28 distinct
transactions = 15 duplicates, against the morning run's 26 distinct after 15
duplicates. Same duplicate count, two more distinct - those messages were
outside the earlier query. Gmail excludes spam/trash without in:anywhere.

Holly only: drawn 5,956.36 -> 6,200.89, current -5,052.58 -> -5,297.11,
projected -2,509.12 -> -2,753.65. Full Team projected 27,462.33 -> 27,217.80.
Earned, Pending and all other people untouched.
</commit_message>
<xml_diff>
--- a/Ampra_Commission_Tracker.xlsx
+++ b/Ampra_Commission_Tracker.xlsx
@@ -773,7 +773,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="31" t="n">
-        <v>5956.36</v>
+        <v>6200.89</v>
       </c>
       <c r="E8" s="31" t="n">
         <v>903.78</v>
@@ -2505,7 +2505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="24" min="1" max="2"/>
@@ -2874,7 +2874,7 @@
     <row r="23" ht="15" customHeight="1" s="25">
       <c r="A23" s="33" t="inlineStr">
         <is>
-          <t>21/08/26</t>
+          <t>23/08/26</t>
         </is>
       </c>
       <c r="B23" s="30" t="inlineStr">
@@ -2884,18 +2884,22 @@
       </c>
       <c r="C23" s="30" t="inlineStr">
         <is>
-          <t>Retainer</t>
+          <t>Meta ad spend (AU)</t>
         </is>
       </c>
       <c r="D23" s="31" t="n">
-        <v>500</v>
-      </c>
-      <c r="E23" s="30" t="n"/>
+        <v>116.59</v>
+      </c>
+      <c r="E23" s="30" t="inlineStr">
+        <is>
+          <t>gross $149.00 less $32.41 Ampra Job (recruitment)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="25">
       <c r="A24" s="33" t="inlineStr">
         <is>
-          <t>20/08/26</t>
+          <t>21/08/26</t>
         </is>
       </c>
       <c r="B24" s="30" t="inlineStr">
@@ -2905,22 +2909,18 @@
       </c>
       <c r="C24" s="30" t="inlineStr">
         <is>
-          <t>Meta ad spend (AU)</t>
+          <t>Retainer</t>
         </is>
       </c>
       <c r="D24" s="31" t="n">
-        <v>37.53</v>
-      </c>
-      <c r="E24" s="30" t="inlineStr">
-        <is>
-          <t>gross $41.58 less $4.05 Ampra Job (recruitment)</t>
-        </is>
-      </c>
+        <v>500</v>
+      </c>
+      <c r="E24" s="30" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
       <c r="A25" s="33" t="inlineStr">
         <is>
-          <t>20/08/26</t>
+          <t>21/08/26</t>
         </is>
       </c>
       <c r="B25" s="30" t="inlineStr">
@@ -2934,18 +2934,18 @@
         </is>
       </c>
       <c r="D25" s="31" t="n">
-        <v>129.64</v>
+        <v>127.94</v>
       </c>
       <c r="E25" s="30" t="inlineStr">
         <is>
-          <t>sub-threshold; billed 19/08 UTC = 20/08 AEST</t>
+          <t>gross $149.00 less $21.06 Ampra Job (recruitment)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="25">
       <c r="A26" s="33" t="inlineStr">
         <is>
-          <t>18/08/26</t>
+          <t>20/08/26</t>
         </is>
       </c>
       <c r="B26" s="30" t="inlineStr">
@@ -2959,14 +2959,18 @@
         </is>
       </c>
       <c r="D26" s="31" t="n">
-        <v>149</v>
-      </c>
-      <c r="E26" s="30" t="n"/>
+        <v>37.53</v>
+      </c>
+      <c r="E26" s="30" t="inlineStr">
+        <is>
+          <t>gross $41.58 less $4.05 Ampra Job (recruitment)</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
       <c r="A27" s="33" t="inlineStr">
         <is>
-          <t>17/08/26</t>
+          <t>20/08/26</t>
         </is>
       </c>
       <c r="B27" s="30" t="inlineStr">
@@ -2976,22 +2980,22 @@
       </c>
       <c r="C27" s="30" t="inlineStr">
         <is>
-          <t>Meta ad spend (NZ)</t>
+          <t>Meta ad spend (AU)</t>
         </is>
       </c>
       <c r="D27" s="31" t="n">
-        <v>252.03</v>
+        <v>129.64</v>
       </c>
       <c r="E27" s="30" t="inlineStr">
         <is>
-          <t>NZ$302.56 at 0.8330 (rate locked at the date struck)</t>
+          <t>sub-threshold; billed 19/08 UTC = 20/08 AEST</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="25">
       <c r="A28" s="33" t="inlineStr">
         <is>
-          <t>16/08/26</t>
+          <t>18/08/26</t>
         </is>
       </c>
       <c r="B28" s="30" t="inlineStr">
@@ -3012,7 +3016,7 @@
     <row r="29" ht="15" customHeight="1" s="25">
       <c r="A29" s="33" t="inlineStr">
         <is>
-          <t>14/08/26</t>
+          <t>17/08/26</t>
         </is>
       </c>
       <c r="B29" s="30" t="inlineStr">
@@ -3022,18 +3026,22 @@
       </c>
       <c r="C29" s="30" t="inlineStr">
         <is>
-          <t>Meta ad spend (AU)</t>
+          <t>Meta ad spend (NZ)</t>
         </is>
       </c>
       <c r="D29" s="31" t="n">
-        <v>149</v>
-      </c>
-      <c r="E29" s="30" t="n"/>
+        <v>252.03</v>
+      </c>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>NZ$302.56 at 0.8330 (rate locked at the date struck)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="25">
       <c r="A30" s="33" t="inlineStr">
         <is>
-          <t>12/08/26</t>
+          <t>16/08/26</t>
         </is>
       </c>
       <c r="B30" s="30" t="inlineStr">
@@ -3054,7 +3062,7 @@
     <row r="31" ht="15" customHeight="1" s="25">
       <c r="A31" s="33" t="inlineStr">
         <is>
-          <t>10/08/26</t>
+          <t>14/08/26</t>
         </is>
       </c>
       <c r="B31" s="30" t="inlineStr">
@@ -3075,48 +3083,44 @@
     <row r="32" ht="15" customHeight="1" s="25">
       <c r="A32" s="33" t="inlineStr">
         <is>
-          <t>09/08/26</t>
+          <t>12/08/26</t>
         </is>
       </c>
       <c r="B32" s="30" t="inlineStr">
         <is>
-          <t>Denzel Winterbeard</t>
+          <t>Holly</t>
         </is>
       </c>
       <c r="C32" s="30" t="inlineStr">
         <is>
-          <t>Retainer</t>
+          <t>Meta ad spend (AU)</t>
         </is>
       </c>
       <c r="D32" s="31" t="n">
-        <v>2500</v>
+        <v>149</v>
       </c>
       <c r="E32" s="30" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="25">
       <c r="A33" s="33" t="inlineStr">
         <is>
-          <t>09/08/26</t>
+          <t>10/08/26</t>
         </is>
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>Hugo</t>
+          <t>Holly</t>
         </is>
       </c>
       <c r="C33" s="30" t="inlineStr">
         <is>
-          <t>Retainer</t>
+          <t>Meta ad spend (AU)</t>
         </is>
       </c>
       <c r="D33" s="31" t="n">
-        <v>1250</v>
-      </c>
-      <c r="E33" s="30" t="inlineStr">
-        <is>
-          <t>Final — ceased on moving to Sales Ops Manager</t>
-        </is>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="E33" s="30" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="25">
       <c r="A34" s="33" t="inlineStr">
@@ -3126,28 +3130,28 @@
       </c>
       <c r="B34" s="30" t="inlineStr">
         <is>
-          <t>Holly</t>
+          <t>Denzel Winterbeard</t>
         </is>
       </c>
       <c r="C34" s="30" t="inlineStr">
         <is>
-          <t>Meta ad spend (AU)</t>
+          <t>Retainer</t>
         </is>
       </c>
       <c r="D34" s="31" t="n">
-        <v>149</v>
+        <v>2500</v>
       </c>
       <c r="E34" s="30" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="25">
       <c r="A35" s="33" t="inlineStr">
         <is>
-          <t>07/08/26</t>
+          <t>09/08/26</t>
         </is>
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>Holly</t>
+          <t>Hugo</t>
         </is>
       </c>
       <c r="C35" s="30" t="inlineStr">
@@ -3156,14 +3160,18 @@
         </is>
       </c>
       <c r="D35" s="31" t="n">
-        <v>500</v>
-      </c>
-      <c r="E35" s="30" t="n"/>
+        <v>1250</v>
+      </c>
+      <c r="E35" s="30" t="inlineStr">
+        <is>
+          <t>Final — ceased on moving to Sales Ops Manager</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="25">
       <c r="A36" s="33" t="inlineStr">
         <is>
-          <t>07/08/26</t>
+          <t>09/08/26</t>
         </is>
       </c>
       <c r="B36" s="30" t="inlineStr">
@@ -3184,7 +3192,7 @@
     <row r="37" ht="15" customHeight="1" s="25">
       <c r="A37" s="33" t="inlineStr">
         <is>
-          <t>05/08/26</t>
+          <t>07/08/26</t>
         </is>
       </c>
       <c r="B37" s="30" t="inlineStr">
@@ -3194,18 +3202,18 @@
       </c>
       <c r="C37" s="30" t="inlineStr">
         <is>
-          <t>Meta ad spend (AU)</t>
+          <t>Retainer</t>
         </is>
       </c>
       <c r="D37" s="31" t="n">
-        <v>149</v>
+        <v>500</v>
       </c>
       <c r="E37" s="30" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
       <c r="A38" s="33" t="inlineStr">
         <is>
-          <t>03/08/26</t>
+          <t>07/08/26</t>
         </is>
       </c>
       <c r="B38" s="30" t="inlineStr">
@@ -3226,7 +3234,7 @@
     <row r="39" ht="15" customHeight="1" s="25">
       <c r="A39" s="33" t="inlineStr">
         <is>
-          <t>02/08/26</t>
+          <t>05/08/26</t>
         </is>
       </c>
       <c r="B39" s="30" t="inlineStr">
@@ -3247,7 +3255,7 @@
     <row r="40" ht="15" customHeight="1" s="25">
       <c r="A40" s="33" t="inlineStr">
         <is>
-          <t>01/08/26</t>
+          <t>03/08/26</t>
         </is>
       </c>
       <c r="B40" s="30" t="inlineStr">
@@ -3268,7 +3276,7 @@
     <row r="41" ht="15" customHeight="1" s="25">
       <c r="A41" s="33" t="inlineStr">
         <is>
-          <t>30/07/26</t>
+          <t>02/08/26</t>
         </is>
       </c>
       <c r="B41" s="30" t="inlineStr">
@@ -3289,7 +3297,7 @@
     <row r="42" ht="15" customHeight="1" s="25">
       <c r="A42" s="33" t="inlineStr">
         <is>
-          <t>29/07/26</t>
+          <t>01/08/26</t>
         </is>
       </c>
       <c r="B42" s="30" t="inlineStr">
@@ -3310,48 +3318,44 @@
     <row r="43" ht="15" customHeight="1" s="25">
       <c r="A43" s="33" t="inlineStr">
         <is>
-          <t>26/07/26</t>
+          <t>30/07/26</t>
         </is>
       </c>
       <c r="B43" s="30" t="inlineStr">
         <is>
-          <t>Denzel Winterbeard</t>
+          <t>Holly</t>
         </is>
       </c>
       <c r="C43" s="30" t="inlineStr">
         <is>
-          <t>Retainer</t>
+          <t>Meta ad spend (AU)</t>
         </is>
       </c>
       <c r="D43" s="31" t="n">
-        <v>2500</v>
+        <v>149</v>
       </c>
       <c r="E43" s="30" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="25">
       <c r="A44" s="33" t="inlineStr">
         <is>
-          <t>26/07/26</t>
+          <t>29/07/26</t>
         </is>
       </c>
       <c r="B44" s="30" t="inlineStr">
         <is>
-          <t>Hugo</t>
+          <t>Holly</t>
         </is>
       </c>
       <c r="C44" s="30" t="inlineStr">
         <is>
-          <t>Retainer</t>
+          <t>Meta ad spend (AU)</t>
         </is>
       </c>
       <c r="D44" s="31" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E44" s="30" t="inlineStr">
-        <is>
-          <t>Two days unpaid leave</t>
-        </is>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="E44" s="30" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="25">
       <c r="A45" s="33" t="inlineStr">
@@ -3361,28 +3365,28 @@
       </c>
       <c r="B45" s="30" t="inlineStr">
         <is>
-          <t>Holly</t>
+          <t>Denzel Winterbeard</t>
         </is>
       </c>
       <c r="C45" s="30" t="inlineStr">
         <is>
-          <t>Meta ad spend (AU)</t>
+          <t>Retainer</t>
         </is>
       </c>
       <c r="D45" s="31" t="n">
-        <v>149</v>
+        <v>2500</v>
       </c>
       <c r="E45" s="30" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="25">
       <c r="A46" s="33" t="inlineStr">
         <is>
-          <t>24/07/26</t>
+          <t>26/07/26</t>
         </is>
       </c>
       <c r="B46" s="30" t="inlineStr">
         <is>
-          <t>Holly</t>
+          <t>Hugo</t>
         </is>
       </c>
       <c r="C46" s="30" t="inlineStr">
@@ -3391,18 +3395,18 @@
         </is>
       </c>
       <c r="D46" s="31" t="n">
-        <v>750</v>
+        <v>2000</v>
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>First draw</t>
+          <t>Two days unpaid leave</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="25">
       <c r="A47" s="33" t="inlineStr">
         <is>
-          <t>24/07/26</t>
+          <t>26/07/26</t>
         </is>
       </c>
       <c r="B47" s="30" t="inlineStr">
@@ -3423,59 +3427,105 @@
     <row r="48" ht="15" customHeight="1" s="25">
       <c r="A48" s="33" t="inlineStr">
         <is>
+          <t>24/07/26</t>
+        </is>
+      </c>
+      <c r="B48" s="30" t="inlineStr">
+        <is>
+          <t>Holly</t>
+        </is>
+      </c>
+      <c r="C48" s="30" t="inlineStr">
+        <is>
+          <t>Retainer</t>
+        </is>
+      </c>
+      <c r="D48" s="31" t="n">
+        <v>750</v>
+      </c>
+      <c r="E48" s="30" t="inlineStr">
+        <is>
+          <t>First draw</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15" customHeight="1" s="25">
+      <c r="A49" s="33" t="inlineStr">
+        <is>
+          <t>24/07/26</t>
+        </is>
+      </c>
+      <c r="B49" s="30" t="inlineStr">
+        <is>
+          <t>Holly</t>
+        </is>
+      </c>
+      <c r="C49" s="30" t="inlineStr">
+        <is>
+          <t>Meta ad spend (AU)</t>
+        </is>
+      </c>
+      <c r="D49" s="31" t="n">
+        <v>149</v>
+      </c>
+      <c r="E49" s="30" t="n"/>
+    </row>
+    <row r="50" ht="15" customHeight="1" s="25">
+      <c r="A50" s="33" t="inlineStr">
+        <is>
           <t>22/07/26</t>
         </is>
       </c>
-      <c r="B48" s="30" t="inlineStr">
+      <c r="B50" s="30" t="inlineStr">
         <is>
           <t>Holly</t>
         </is>
       </c>
-      <c r="C48" s="30" t="inlineStr">
+      <c r="C50" s="30" t="inlineStr">
         <is>
           <t>Meta ad spend (AU)</t>
         </is>
       </c>
-      <c r="D48" s="31" t="n">
+      <c r="D50" s="31" t="n">
         <v>149</v>
       </c>
-      <c r="E48" s="30" t="inlineStr">
+      <c r="E50" s="30" t="inlineStr">
         <is>
           <t>billing period 19/07–22/07 straddles the 20/07 baseline — included in full</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="15" customHeight="1" s="25">
-      <c r="A49" s="34" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="34" t="inlineStr">
         <is>
           <t>TOTAL DRAWN</t>
         </is>
       </c>
-      <c r="B49" s="44" t="n"/>
-      <c r="C49" s="44" t="n"/>
-      <c r="D49" s="35">
-        <f>SUM(D13:D48)</f>
-        <v/>
-      </c>
-      <c r="E49" s="44" t="inlineStr">
+      <c r="B51" s="44" t="n"/>
+      <c r="C51" s="44" t="n"/>
+      <c r="D51" s="35">
+        <f>SUM(D13:D50)</f>
+        <v/>
+      </c>
+      <c r="E51" s="44" t="inlineStr">
         <is>
           <t>Must equal the Dashboard 'Retainer + Ad Spend' total</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="15" customHeight="1" s="25">
-      <c r="A50" s="34" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="34" t="inlineStr">
         <is>
           <t>CHECK</t>
         </is>
       </c>
-      <c r="B50" s="44" t="n"/>
-      <c r="C50" s="44" t="n"/>
-      <c r="D50" s="35">
-        <f>D49-'📊 Dashboard'!D10</f>
-        <v/>
-      </c>
-      <c r="E50" s="44" t="inlineStr">
+      <c r="B52" s="44" t="n"/>
+      <c r="C52" s="44" t="n"/>
+      <c r="D52" s="35">
+        <f>D51-'📊 Dashboard'!D10</f>
+        <v/>
+      </c>
+      <c r="E52" s="44" t="inlineStr">
         <is>
           <t>Zero means the two tabs agree</t>
         </is>

</xml_diff>